<commit_message>
edit in cold store
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/hawa huri jhyal/hawa huri jhyal 2082_2083.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/hawa huri jhyal/hawa huri jhyal 2082_2083.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\बजेट माग estimate\nagar bhaipari and estimate misc\hawa huri jhyal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{276E0937-9F04-4223-B03E-361861839426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB31C8EF-E4EE-44A3-B027-2521CF3604FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="212">
   <si>
     <t>S.N.</t>
   </si>
@@ -1020,6 +1020,9 @@
   </si>
   <si>
     <t>Date: 2083/03/18</t>
+  </si>
+  <si>
+    <t>Detail Valuated Sheet</t>
   </si>
 </sst>
 </file>
@@ -3572,6 +3575,21 @@
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="32" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="32" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="32" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3588,21 +3606,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="65" fillId="32" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="65" fillId="32" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="65" fillId="32" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="51" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6891,7 +6894,7 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="184" t="s">
-        <v>22</v>
+        <v>211</v>
       </c>
       <c r="B4" s="184"/>
       <c r="C4" s="184"/>
@@ -7744,7 +7747,7 @@
       <c r="I43" s="129"/>
       <c r="J43" s="130"/>
       <c r="K43" s="150">
-        <f>SUM(K9:K42)</f>
+        <f>SUM(K10:K42)</f>
         <v>48124.74305248</v>
       </c>
       <c r="L43" s="151"/>
@@ -8759,60 +8762,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="188" t="s">
+      <c r="A1" s="193" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="188"/>
-      <c r="C1" s="188"/>
-      <c r="D1" s="188"/>
-      <c r="E1" s="188"/>
-      <c r="F1" s="188"/>
-      <c r="G1" s="188"/>
-      <c r="H1" s="188"/>
-      <c r="I1" s="188"/>
-      <c r="J1" s="188"/>
+      <c r="B1" s="193"/>
+      <c r="C1" s="193"/>
+      <c r="D1" s="193"/>
+      <c r="E1" s="193"/>
+      <c r="F1" s="193"/>
+      <c r="G1" s="193"/>
+      <c r="H1" s="193"/>
+      <c r="I1" s="193"/>
+      <c r="J1" s="193"/>
     </row>
     <row r="2" spans="1:10" ht="25.5">
-      <c r="A2" s="189" t="s">
+      <c r="A2" s="194" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="189"/>
-      <c r="C2" s="189"/>
-      <c r="D2" s="189"/>
-      <c r="E2" s="189"/>
-      <c r="F2" s="189"/>
-      <c r="G2" s="189"/>
-      <c r="H2" s="189"/>
-      <c r="I2" s="189"/>
-      <c r="J2" s="189"/>
+      <c r="B2" s="194"/>
+      <c r="C2" s="194"/>
+      <c r="D2" s="194"/>
+      <c r="E2" s="194"/>
+      <c r="F2" s="194"/>
+      <c r="G2" s="194"/>
+      <c r="H2" s="194"/>
+      <c r="I2" s="194"/>
+      <c r="J2" s="194"/>
     </row>
     <row r="3" spans="1:10" ht="18.75">
-      <c r="A3" s="190" t="s">
+      <c r="A3" s="195" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="190"/>
-      <c r="C3" s="190"/>
-      <c r="D3" s="190"/>
-      <c r="E3" s="190"/>
-      <c r="F3" s="190"/>
-      <c r="G3" s="190"/>
-      <c r="H3" s="190"/>
-      <c r="I3" s="190"/>
-      <c r="J3" s="190"/>
+      <c r="B3" s="195"/>
+      <c r="C3" s="195"/>
+      <c r="D3" s="195"/>
+      <c r="E3" s="195"/>
+      <c r="F3" s="195"/>
+      <c r="G3" s="195"/>
+      <c r="H3" s="195"/>
+      <c r="I3" s="195"/>
+      <c r="J3" s="195"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="191" t="s">
+      <c r="A4" s="196" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="191"/>
-      <c r="C4" s="191"/>
-      <c r="D4" s="191"/>
-      <c r="E4" s="191"/>
-      <c r="F4" s="191"/>
-      <c r="G4" s="191"/>
-      <c r="H4" s="191"/>
-      <c r="I4" s="191"/>
-      <c r="J4" s="191"/>
+      <c r="B4" s="196"/>
+      <c r="C4" s="196"/>
+      <c r="D4" s="196"/>
+      <c r="E4" s="196"/>
+      <c r="F4" s="196"/>
+      <c r="G4" s="196"/>
+      <c r="H4" s="196"/>
+      <c r="I4" s="196"/>
+      <c r="J4" s="196"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="37"/>
@@ -8831,33 +8834,33 @@
         <v>55</v>
       </c>
       <c r="B6" s="31"/>
-      <c r="C6" s="192" t="e">
+      <c r="C6" s="197" t="e">
         <f>E51</f>
         <v>#REF!</v>
       </c>
-      <c r="D6" s="193"/>
+      <c r="D6" s="198"/>
       <c r="E6" s="31"/>
       <c r="F6" s="31"/>
       <c r="G6" s="31" t="s">
         <v>56</v>
       </c>
       <c r="H6" s="31"/>
-      <c r="I6" s="192" t="e">
+      <c r="I6" s="197" t="e">
         <f>H51</f>
         <v>#REF!</v>
       </c>
-      <c r="J6" s="193"/>
+      <c r="J6" s="198"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="32"/>
       <c r="B7" s="32"/>
-      <c r="C7" s="194"/>
-      <c r="D7" s="194"/>
-      <c r="E7" s="194"/>
-      <c r="F7" s="194"/>
-      <c r="H7" s="195"/>
-      <c r="I7" s="195"/>
-      <c r="J7" s="195"/>
+      <c r="C7" s="188"/>
+      <c r="D7" s="188"/>
+      <c r="E7" s="188"/>
+      <c r="F7" s="188"/>
+      <c r="H7" s="189"/>
+      <c r="I7" s="189"/>
+      <c r="J7" s="189"/>
     </row>
     <row r="8" spans="1:10" ht="16.5">
       <c r="A8" t="s">
@@ -8884,32 +8887,32 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="196" t="s">
+      <c r="A10" s="190" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="196" t="s">
+      <c r="B10" s="190" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="198" t="s">
+      <c r="C10" s="192" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="198"/>
-      <c r="E10" s="198"/>
-      <c r="F10" s="198" t="s">
+      <c r="D10" s="192"/>
+      <c r="E10" s="192"/>
+      <c r="F10" s="192" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="198"/>
-      <c r="H10" s="198"/>
-      <c r="I10" s="196" t="s">
+      <c r="G10" s="192"/>
+      <c r="H10" s="192"/>
+      <c r="I10" s="190" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="196" t="s">
+      <c r="J10" s="190" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="197"/>
-      <c r="B11" s="197"/>
+      <c r="A11" s="191"/>
+      <c r="B11" s="191"/>
       <c r="C11" s="39" t="s">
         <v>64</v>
       </c>
@@ -8928,8 +8931,8 @@
       <c r="H11" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="I11" s="197"/>
-      <c r="J11" s="197"/>
+      <c r="I11" s="191"/>
+      <c r="J11" s="191"/>
     </row>
     <row r="12" spans="1:10" ht="15.75">
       <c r="A12" s="47">
@@ -9856,6 +9859,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="H7:J7"/>
@@ -9865,12 +9874,6 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I10:I11"/>
     <mergeCell ref="J10:J11"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -13251,6 +13254,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="D161:E161"/>
+    <mergeCell ref="D162:E162"/>
+    <mergeCell ref="D156:E156"/>
+    <mergeCell ref="D157:E157"/>
+    <mergeCell ref="D158:E158"/>
+    <mergeCell ref="D159:E159"/>
+    <mergeCell ref="D160:E160"/>
     <mergeCell ref="B6:G6"/>
     <mergeCell ref="I6:L6"/>
     <mergeCell ref="A1:L1"/>
@@ -13258,13 +13268,6 @@
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="K5:L5"/>
-    <mergeCell ref="D161:E161"/>
-    <mergeCell ref="D162:E162"/>
-    <mergeCell ref="D156:E156"/>
-    <mergeCell ref="D157:E157"/>
-    <mergeCell ref="D158:E158"/>
-    <mergeCell ref="D159:E159"/>
-    <mergeCell ref="D160:E160"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
jhyal dhoka hawa huri edit
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/hawa huri jhyal/hawa huri jhyal 2082_2083.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/hawa huri jhyal/hawa huri jhyal 2082_2083.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\बजेट माग estimate\nagar bhaipari and estimate misc\hawa huri jhyal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB31C8EF-E4EE-44A3-B027-2521CF3604FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74AD889A-6D46-4AAA-8E38-E785376CEB9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="213">
   <si>
     <t>S.N.</t>
   </si>
@@ -1023,6 +1023,9 @@
   </si>
   <si>
     <t>Detail Valuated Sheet</t>
+  </si>
+  <si>
+    <t>Total Valuated</t>
   </si>
 </sst>
 </file>
@@ -3575,6 +3578,24 @@
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="63" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3588,24 +3609,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="65" fillId="32" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="63" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="51" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -7686,11 +7689,11 @@
         <v>163</v>
       </c>
       <c r="J40" s="178">
-        <v>25000</v>
+        <v>26000</v>
       </c>
       <c r="K40" s="178">
         <f>H40*J40</f>
-        <v>25000</v>
+        <v>26000</v>
       </c>
       <c r="L40" s="179"/>
     </row>
@@ -7748,7 +7751,7 @@
       <c r="J43" s="130"/>
       <c r="K43" s="150">
         <f>SUM(K10:K42)</f>
-        <v>48124.74305248</v>
+        <v>49124.74305248</v>
       </c>
       <c r="L43" s="151"/>
     </row>
@@ -7766,11 +7769,11 @@
     </row>
     <row r="45" spans="2:12">
       <c r="C45" s="134" t="s">
-        <v>13</v>
+        <v>212</v>
       </c>
       <c r="D45" s="180">
         <f>+K43</f>
-        <v>48124.74305248</v>
+        <v>49124.74305248</v>
       </c>
       <c r="E45" s="180"/>
       <c r="G45" s="64"/>
@@ -7783,7 +7786,7 @@
       </c>
       <c r="D46" s="180">
         <f>13%*D45</f>
-        <v>6256.2165968223999</v>
+        <v>6386.2165968223999</v>
       </c>
       <c r="E46" s="180"/>
       <c r="G46" s="64"/>
@@ -7796,7 +7799,7 @@
       </c>
       <c r="D47" s="180">
         <f>SUM(D45:E46)</f>
-        <v>54380.9596493024</v>
+        <v>55510.9596493024</v>
       </c>
       <c r="E47" s="181"/>
       <c r="G47" s="62"/>
@@ -8762,60 +8765,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="193" t="s">
+      <c r="A1" s="188" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="193"/>
-      <c r="C1" s="193"/>
-      <c r="D1" s="193"/>
-      <c r="E1" s="193"/>
-      <c r="F1" s="193"/>
-      <c r="G1" s="193"/>
-      <c r="H1" s="193"/>
-      <c r="I1" s="193"/>
-      <c r="J1" s="193"/>
+      <c r="B1" s="188"/>
+      <c r="C1" s="188"/>
+      <c r="D1" s="188"/>
+      <c r="E1" s="188"/>
+      <c r="F1" s="188"/>
+      <c r="G1" s="188"/>
+      <c r="H1" s="188"/>
+      <c r="I1" s="188"/>
+      <c r="J1" s="188"/>
     </row>
     <row r="2" spans="1:10" ht="25.5">
-      <c r="A2" s="194" t="s">
+      <c r="A2" s="189" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="194"/>
-      <c r="C2" s="194"/>
-      <c r="D2" s="194"/>
-      <c r="E2" s="194"/>
-      <c r="F2" s="194"/>
-      <c r="G2" s="194"/>
-      <c r="H2" s="194"/>
-      <c r="I2" s="194"/>
-      <c r="J2" s="194"/>
+      <c r="B2" s="189"/>
+      <c r="C2" s="189"/>
+      <c r="D2" s="189"/>
+      <c r="E2" s="189"/>
+      <c r="F2" s="189"/>
+      <c r="G2" s="189"/>
+      <c r="H2" s="189"/>
+      <c r="I2" s="189"/>
+      <c r="J2" s="189"/>
     </row>
     <row r="3" spans="1:10" ht="18.75">
-      <c r="A3" s="195" t="s">
+      <c r="A3" s="190" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="195"/>
-      <c r="C3" s="195"/>
-      <c r="D3" s="195"/>
-      <c r="E3" s="195"/>
-      <c r="F3" s="195"/>
-      <c r="G3" s="195"/>
-      <c r="H3" s="195"/>
-      <c r="I3" s="195"/>
-      <c r="J3" s="195"/>
+      <c r="B3" s="190"/>
+      <c r="C3" s="190"/>
+      <c r="D3" s="190"/>
+      <c r="E3" s="190"/>
+      <c r="F3" s="190"/>
+      <c r="G3" s="190"/>
+      <c r="H3" s="190"/>
+      <c r="I3" s="190"/>
+      <c r="J3" s="190"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="196" t="s">
+      <c r="A4" s="191" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="196"/>
-      <c r="C4" s="196"/>
-      <c r="D4" s="196"/>
-      <c r="E4" s="196"/>
-      <c r="F4" s="196"/>
-      <c r="G4" s="196"/>
-      <c r="H4" s="196"/>
-      <c r="I4" s="196"/>
-      <c r="J4" s="196"/>
+      <c r="B4" s="191"/>
+      <c r="C4" s="191"/>
+      <c r="D4" s="191"/>
+      <c r="E4" s="191"/>
+      <c r="F4" s="191"/>
+      <c r="G4" s="191"/>
+      <c r="H4" s="191"/>
+      <c r="I4" s="191"/>
+      <c r="J4" s="191"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="37"/>
@@ -8834,33 +8837,33 @@
         <v>55</v>
       </c>
       <c r="B6" s="31"/>
-      <c r="C6" s="197" t="e">
+      <c r="C6" s="192" t="e">
         <f>E51</f>
         <v>#REF!</v>
       </c>
-      <c r="D6" s="198"/>
+      <c r="D6" s="193"/>
       <c r="E6" s="31"/>
       <c r="F6" s="31"/>
       <c r="G6" s="31" t="s">
         <v>56</v>
       </c>
       <c r="H6" s="31"/>
-      <c r="I6" s="197" t="e">
+      <c r="I6" s="192" t="e">
         <f>H51</f>
         <v>#REF!</v>
       </c>
-      <c r="J6" s="198"/>
+      <c r="J6" s="193"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="32"/>
       <c r="B7" s="32"/>
-      <c r="C7" s="188"/>
-      <c r="D7" s="188"/>
-      <c r="E7" s="188"/>
-      <c r="F7" s="188"/>
-      <c r="H7" s="189"/>
-      <c r="I7" s="189"/>
-      <c r="J7" s="189"/>
+      <c r="C7" s="194"/>
+      <c r="D7" s="194"/>
+      <c r="E7" s="194"/>
+      <c r="F7" s="194"/>
+      <c r="H7" s="195"/>
+      <c r="I7" s="195"/>
+      <c r="J7" s="195"/>
     </row>
     <row r="8" spans="1:10" ht="16.5">
       <c r="A8" t="s">
@@ -8887,32 +8890,32 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="190" t="s">
+      <c r="A10" s="196" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="190" t="s">
+      <c r="B10" s="196" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="192" t="s">
+      <c r="C10" s="198" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="192"/>
-      <c r="E10" s="192"/>
-      <c r="F10" s="192" t="s">
+      <c r="D10" s="198"/>
+      <c r="E10" s="198"/>
+      <c r="F10" s="198" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="192"/>
-      <c r="H10" s="192"/>
-      <c r="I10" s="190" t="s">
+      <c r="G10" s="198"/>
+      <c r="H10" s="198"/>
+      <c r="I10" s="196" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="190" t="s">
+      <c r="J10" s="196" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="191"/>
-      <c r="B11" s="191"/>
+      <c r="A11" s="197"/>
+      <c r="B11" s="197"/>
       <c r="C11" s="39" t="s">
         <v>64</v>
       </c>
@@ -8931,8 +8934,8 @@
       <c r="H11" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="I11" s="191"/>
-      <c r="J11" s="191"/>
+      <c r="I11" s="197"/>
+      <c r="J11" s="197"/>
     </row>
     <row r="12" spans="1:10" ht="15.75">
       <c r="A12" s="47">
@@ -9859,12 +9862,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="I6:J6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="H7:J7"/>
@@ -9874,6 +9871,12 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I10:I11"/>
     <mergeCell ref="J10:J11"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -13254,6 +13257,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="K5:L5"/>
     <mergeCell ref="D161:E161"/>
     <mergeCell ref="D162:E162"/>
     <mergeCell ref="D156:E156"/>
@@ -13261,13 +13271,6 @@
     <mergeCell ref="D158:E158"/>
     <mergeCell ref="D159:E159"/>
     <mergeCell ref="D160:E160"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="I6:L6"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="K5:L5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>